<commit_message>
feat(phase3): 完成 Actions 工作流 Runner 与 required-check 联动
- WorkflowRunner：shell/python/http 步骤执行器
- WorkflowTrigger：运行记录 + 审计/trace 留痕
- WorkflowCheck：required-check 拦截失败工作流后的 PR 合并
- gx workflow run/list 子命令与种子 ci-check 工作流
- 工作流单元/集成测试
</commit_message>
<xml_diff>
--- a/demo/seed-workbook.xlsx
+++ b/demo/seed-workbook.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-31T15:07:29.224363Z</t>
+          <t>2026-08-31T16:28:57.566660Z</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-31T15:07:29.265891Z</t>
+          <t>2026-08-31T16:28:57.603530Z</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -642,6 +642,31 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ci-check</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>[{"type": "shell", "command": "echo ok"}]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>active</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add demo trace output for gosim preliminary
</commit_message>
<xml_diff>
--- a/demo/seed-workbook.xlsx
+++ b/demo/seed-workbook.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-31T16:28:57.566660Z</t>
+          <t>2026-09-01T15:40:35.119438Z</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-31T16:28:57.603530Z</t>
+          <t>2026-09-01T15:40:35.144122Z</t>
         </is>
       </c>
     </row>

</xml_diff>